<commit_message>
Updated negative test validation
</commit_message>
<xml_diff>
--- a/rules/CORE-000011/negative/01/data/unit-test-coreid-CG0175-negative.xlsx
+++ b/rules/CORE-000011/negative/01/data/unit-test-coreid-CG0175-negative.xlsx
@@ -559,10 +559,10 @@
         <v>5</v>
       </c>
       <c r="E2" s="2" t="str">
-        <v>IECAT</v>
+        <v>IEORRES</v>
       </c>
       <c r="F2" s="2" t="str">
-        <v>EXCLUSION</v>
+        <v>N</v>
       </c>
     </row>
     <row r="3">
@@ -579,10 +579,10 @@
         <v>5</v>
       </c>
       <c r="E3" s="2" t="str">
-        <v>IEORRES</v>
+        <v>IECAT</v>
       </c>
       <c r="F3" s="2" t="str">
-        <v>N</v>
+        <v>EXCLUSION</v>
       </c>
     </row>
   </sheetData>

</xml_diff>